<commit_message>
W29 2026 update #2 (55 stocks, 7/14 lists, industries in Chinese)
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -471,24 +471,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1347 HK</t>
+          <t>2359 HK</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>华虹宏力</t>
+          <t>药明康德</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>诊断与研究</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.68</v>
+        <v>0.82</v>
       </c>
       <c r="F2" t="n">
-        <v>0.58</v>
+        <v>0.72</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -499,7 +499,7 @@
         <v>1.01</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2871</v>
+        <v>0.1316</v>
       </c>
     </row>
     <row r="3">
@@ -510,24 +510,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>992 HK</t>
+          <t>2269 HK</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>联想集团</t>
+          <t>药明生物</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Computer Hardware</t>
+          <t>生物科技</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.74</v>
+        <v>0.82</v>
       </c>
       <c r="F3" t="n">
-        <v>0.64</v>
+        <v>0.72</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
         <v>1.01</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1669</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="4">
@@ -549,24 +549,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2359 HK</t>
+          <t>1024 HK</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>药明康德</t>
+          <t>快手-W</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Diagnostics &amp; Research</t>
+          <t>互联网内容与信息</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         <v>1.01</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1392</v>
+        <v>0.177</v>
       </c>
     </row>
     <row r="5">
@@ -588,24 +588,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>522 HK</t>
+          <t>2382 HK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASMPT</t>
+          <t>舜宇光学</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment &amp; Materials</t>
+          <t>光学/AI硬件</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.71</v>
+        <v>0.84</v>
       </c>
       <c r="F5" t="n">
-        <v>0.61</v>
+        <v>0.74</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>1.01</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1812</v>
+        <v>0.2291</v>
       </c>
     </row>
     <row r="6">
@@ -627,24 +627,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2269 HK</t>
+          <t>763 HK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>药明生物</t>
+          <t>中兴通讯</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Biotechnology</t>
+          <t>通信设备</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="F6" t="n">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
         <v>1.01</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1796</v>
+        <v>0.1717</v>
       </c>
     </row>
     <row r="7">
@@ -666,24 +666,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2338 HK</t>
+          <t>9988 HK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>潍柴动力</t>
+          <t>阿里巴巴</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Auto Manufacturers</t>
+          <t>电商/云</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
         <v>1.01</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1536</v>
+        <v>0.1398</v>
       </c>
     </row>
     <row r="8">
@@ -719,10 +719,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
       <c r="F8" t="n">
-        <v>0.52</v>
+        <v>0.55</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         <v>1.01</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2751</v>
+        <v>0.2832</v>
       </c>
     </row>
     <row r="9">
@@ -772,7 +772,7 @@
         <v>1.01</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2673</v>
+        <v>0.2692</v>
       </c>
     </row>
     <row r="10">
@@ -793,7 +793,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Electronic Components</t>
+          <t>电子元件</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -811,7 +811,7 @@
         <v>1.01</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2733</v>
+        <v>0.2778</v>
       </c>
     </row>
     <row r="11">
@@ -822,24 +822,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TSM US</t>
+          <t>TXN US</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>台积电ADR</t>
+          <t>德州仪器</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>晶圆代工</t>
+          <t>半导体</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="F11" t="n">
-        <v>0.73</v>
+        <v>0.68</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>1.01</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1867</v>
+        <v>0.1983</v>
       </c>
     </row>
     <row r="12">
@@ -861,24 +861,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TXN US</t>
+          <t>TSM US</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>德州仪器</t>
+          <t>台积电ADR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>晶圆代工</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.79</v>
+        <v>0.84</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.74</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         <v>1.01</v>
       </c>
       <c r="I12" t="n">
-        <v>0.2193</v>
+        <v>0.1935</v>
       </c>
     </row>
     <row r="13">
@@ -900,24 +900,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>APH US</t>
+          <t>CSCO US</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>安费诺</t>
+          <t>思科</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Electronic Components</t>
+          <t>通信设备</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F13" t="n">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1.01</v>
       </c>
       <c r="I13" t="n">
-        <v>0.2122</v>
+        <v>0.164</v>
       </c>
     </row>
     <row r="14">
@@ -939,24 +939,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CSCO US</t>
+          <t>ADI US</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>思科</t>
+          <t>亚德诺</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Communication Equipment</t>
+          <t>半导体</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F14" t="n">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
         <v>1.01</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1602</v>
+        <v>0.2065</v>
       </c>
     </row>
     <row r="15">
@@ -1006,7 +1006,7 @@
         <v>1.01</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1201</v>
+        <v>0.1189</v>
       </c>
     </row>
     <row r="16">
@@ -1017,24 +1017,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ADI US</t>
+          <t>APH US</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>亚德诺</t>
+          <t>安费诺</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>电子元件</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="F16" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         <v>1.01</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2045</v>
+        <v>0.2043</v>
       </c>
     </row>
     <row r="17">
@@ -1056,24 +1056,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AVGO US</t>
+          <t>CAT US</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>博通</t>
+          <t>卡特彼勒</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>半导体</t>
+          <t>农业与重型工程机械</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         <v>1.01</v>
       </c>
       <c r="I17" t="n">
-        <v>0.21</v>
+        <v>0.1525</v>
       </c>
     </row>
     <row r="18">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NVDA US</t>
+          <t>META US</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI芯片</t>
+          <t>广告/AI</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F18" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
         <v>1.01</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1485</v>
+        <v>0.1408</v>
       </c>
     </row>
     <row r="19">
@@ -1134,24 +1134,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CAT US</t>
+          <t>AVGO US</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>卡特彼勒</t>
+          <t>博通</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Farm &amp; Heavy Construction Machinery</t>
+          <t>半导体</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="F19" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>1.01</v>
       </c>
       <c r="I19" t="n">
-        <v>0.164</v>
+        <v>0.2012</v>
       </c>
     </row>
     <row r="20">
@@ -1173,24 +1173,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>VST US</t>
+          <t>NVDA US</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Vistra Energy</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Utilities - Independent Power Producers</t>
+          <t>AI芯片</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F20" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
         <v>1.01</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1936</v>
+        <v>0.1494</v>
       </c>
     </row>
     <row r="21">
@@ -1212,24 +1212,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MELI US</t>
+          <t>VST US</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MercadoLibre</t>
+          <t>Vistra Energy</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Internet Retail</t>
+          <t>独立发电商</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F21" t="n">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1697</v>
+        <v>0.1883</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W30 2026 weekly update (57 stocks)
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -2,27 +2,33 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <sz val="9"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -46,11 +52,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -414,7 +421,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
+  <cols>
+    <col width="9.5" bestFit="1" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -485,10 +495,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -498,8 +508,8 @@
       <c r="H2" t="n">
         <v>1.01</v>
       </c>
-      <c r="I2" t="n">
-        <v>0.1316</v>
+      <c r="I2" s="1" t="n">
+        <v>0.1419</v>
       </c>
     </row>
     <row r="3">
@@ -524,10 +534,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="F3" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -537,8 +547,8 @@
       <c r="H3" t="n">
         <v>1.01</v>
       </c>
-      <c r="I3" t="n">
-        <v>0.18</v>
+      <c r="I3" s="1" t="n">
+        <v>0.1901</v>
       </c>
     </row>
     <row r="4">
@@ -563,10 +573,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="F4" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -576,8 +586,8 @@
       <c r="H4" t="n">
         <v>1.01</v>
       </c>
-      <c r="I4" t="n">
-        <v>0.177</v>
+      <c r="I4" s="1" t="n">
+        <v>0.2025</v>
       </c>
     </row>
     <row r="5">
@@ -588,24 +598,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2382 HK</t>
+          <t>9626 HK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>舜宇光学</t>
+          <t>哔哩哔哩</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>光学/AI硬件</t>
+          <t>视频社区</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="F5" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -615,8 +625,8 @@
       <c r="H5" t="n">
         <v>1.01</v>
       </c>
-      <c r="I5" t="n">
-        <v>0.2291</v>
+      <c r="I5" s="1" t="n">
+        <v>0.2017</v>
       </c>
     </row>
     <row r="6">
@@ -627,24 +637,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>763 HK</t>
+          <t>2382 HK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>中兴通讯</t>
+          <t>舜宇光学</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>通信设备</t>
+          <t>光学/AI硬件</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -654,8 +664,8 @@
       <c r="H6" t="n">
         <v>1.01</v>
       </c>
-      <c r="I6" t="n">
-        <v>0.1717</v>
+      <c r="I6" s="1" t="n">
+        <v>0.2033</v>
       </c>
     </row>
     <row r="7">
@@ -680,10 +690,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="F7" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -693,8 +703,8 @@
       <c r="H7" t="n">
         <v>1.01</v>
       </c>
-      <c r="I7" t="n">
-        <v>0.1398</v>
+      <c r="I7" s="1" t="n">
+        <v>0.1557</v>
       </c>
     </row>
     <row r="8">
@@ -705,24 +715,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MU US</t>
+          <t>TSM US</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>美光</t>
+          <t>台积电ADR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>内存/HBM</t>
+          <t>晶圆代工</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.65</v>
+        <v>0.79</v>
       </c>
       <c r="F8" t="n">
-        <v>0.55</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -732,8 +742,8 @@
       <c r="H8" t="n">
         <v>1.01</v>
       </c>
-      <c r="I8" t="n">
-        <v>0.2832</v>
+      <c r="I8" s="1" t="n">
+        <v>0.155</v>
       </c>
     </row>
     <row r="9">
@@ -744,24 +754,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AMD US</t>
+          <t>TXN US</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>德州仪器</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI芯片</t>
+          <t>半导体</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.74</v>
+        <v>0.78</v>
       </c>
       <c r="F9" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -771,8 +781,8 @@
       <c r="H9" t="n">
         <v>1.01</v>
       </c>
-      <c r="I9" t="n">
-        <v>0.2692</v>
+      <c r="I9" s="1" t="n">
+        <v>0.2129</v>
       </c>
     </row>
     <row r="10">
@@ -783,24 +793,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GLW US</t>
+          <t>LLY US</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>康宁</t>
+          <t>礼来</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>电子元件</t>
+          <t>制药</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.68</v>
+        <v>0.85</v>
       </c>
       <c r="F10" t="n">
-        <v>0.58</v>
+        <v>0.75</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -810,8 +820,8 @@
       <c r="H10" t="n">
         <v>1.01</v>
       </c>
-      <c r="I10" t="n">
-        <v>0.2778</v>
+      <c r="I10" s="1" t="n">
+        <v>0.1323</v>
       </c>
     </row>
     <row r="11">
@@ -822,24 +832,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TXN US</t>
+          <t>APH US</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>德州仪器</t>
+          <t>安费诺</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>半导体</t>
+          <t>电子元件</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.78</v>
+        <v>0.82</v>
       </c>
       <c r="F11" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -849,8 +859,8 @@
       <c r="H11" t="n">
         <v>1.01</v>
       </c>
-      <c r="I11" t="n">
-        <v>0.1983</v>
+      <c r="I11" s="1" t="n">
+        <v>0.2232</v>
       </c>
     </row>
     <row r="12">
@@ -861,24 +871,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TSM US</t>
+          <t>CSCO US</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>台积电ADR</t>
+          <t>思科</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>晶圆代工</t>
+          <t>通信设备</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="F12" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -888,8 +898,8 @@
       <c r="H12" t="n">
         <v>1.01</v>
       </c>
-      <c r="I12" t="n">
-        <v>0.1935</v>
+      <c r="I12" s="1" t="n">
+        <v>0.1588</v>
       </c>
     </row>
     <row r="13">
@@ -900,17 +910,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CSCO US</t>
+          <t>HWM US</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>思科</t>
+          <t>Howmet Aerospace</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>通信设备</t>
+          <t>航空航天与国防</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -927,8 +937,8 @@
       <c r="H13" t="n">
         <v>1.01</v>
       </c>
-      <c r="I13" t="n">
-        <v>0.164</v>
+      <c r="I13" s="1" t="n">
+        <v>0.1374</v>
       </c>
     </row>
     <row r="14">
@@ -939,24 +949,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ADI US</t>
+          <t>CAT US</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>亚德诺</t>
+          <t>卡特彼勒</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>半导体</t>
+          <t>农业与重型工程机械</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="F14" t="n">
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -966,8 +976,8 @@
       <c r="H14" t="n">
         <v>1.01</v>
       </c>
-      <c r="I14" t="n">
-        <v>0.2065</v>
+      <c r="I14" s="1" t="n">
+        <v>0.1668</v>
       </c>
     </row>
     <row r="15">
@@ -978,24 +988,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LLY US</t>
+          <t>NVDA US</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>礼来</t>
+          <t>英伟达</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>制药</t>
+          <t>AI芯片</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F15" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1005,8 +1015,8 @@
       <c r="H15" t="n">
         <v>1.01</v>
       </c>
-      <c r="I15" t="n">
-        <v>0.1189</v>
+      <c r="I15" s="1" t="n">
+        <v>0.1664</v>
       </c>
     </row>
     <row r="16">
@@ -1017,17 +1027,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>APH US</t>
+          <t>ADI US</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>安费诺</t>
+          <t>亚德诺</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>电子元件</t>
+          <t>半导体</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1044,8 +1054,8 @@
       <c r="H16" t="n">
         <v>1.01</v>
       </c>
-      <c r="I16" t="n">
-        <v>0.2043</v>
+      <c r="I16" s="1" t="n">
+        <v>0.2118</v>
       </c>
     </row>
     <row r="17">
@@ -1056,24 +1066,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CAT US</t>
+          <t>META US</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>卡特彼勒</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>农业与重型工程机械</t>
+          <t>广告/AI</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="F17" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1083,8 +1093,8 @@
       <c r="H17" t="n">
         <v>1.01</v>
       </c>
-      <c r="I17" t="n">
-        <v>0.1525</v>
+      <c r="I17" s="1" t="n">
+        <v>0.1541</v>
       </c>
     </row>
     <row r="18">
@@ -1095,24 +1105,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>META US</t>
+          <t>AVGO US</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>博通</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>广告/AI</t>
+          <t>半导体</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="F18" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1122,8 +1132,8 @@
       <c r="H18" t="n">
         <v>1.01</v>
       </c>
-      <c r="I18" t="n">
-        <v>0.1408</v>
+      <c r="I18" s="1" t="n">
+        <v>0.2195</v>
       </c>
     </row>
     <row r="19">
@@ -1134,24 +1144,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AVGO US</t>
+          <t>NOW US</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>博通</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>半导体</t>
+          <t>AI软件</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.83</v>
+        <v>0.76</v>
       </c>
       <c r="F19" t="n">
-        <v>0.73</v>
+        <v>0.66</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1161,8 +1171,8 @@
       <c r="H19" t="n">
         <v>1.01</v>
       </c>
-      <c r="I19" t="n">
-        <v>0.2012</v>
+      <c r="I19" s="1" t="n">
+        <v>0.2195</v>
       </c>
     </row>
     <row r="20">
@@ -1173,17 +1183,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NVDA US</t>
+          <t>MELI US</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>英伟达</t>
+          <t>MercadoLibre</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AI芯片</t>
+          <t>互联网零售</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1200,8 +1210,8 @@
       <c r="H20" t="n">
         <v>1.01</v>
       </c>
-      <c r="I20" t="n">
-        <v>0.1494</v>
+      <c r="I20" s="1" t="n">
+        <v>0.146</v>
       </c>
     </row>
     <row r="21">
@@ -1212,24 +1222,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VST US</t>
+          <t>INTU US</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Vistra Energy</t>
+          <t>财捷</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>独立发电商</t>
+          <t>应用软件</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="F21" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1239,8 +1249,8 @@
       <c r="H21" t="n">
         <v>1.01</v>
       </c>
-      <c r="I21" t="n">
-        <v>0.1883</v>
+      <c r="I21" s="1" t="n">
+        <v>0.2172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>